<commit_message>
Update oil list with Liqui Moly oils
</commit_message>
<xml_diff>
--- a/OelExport/Artikel.XLSX
+++ b/OelExport/Artikel.XLSX
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409">
   <si>
     <t>Status</t>
   </si>
@@ -161,7 +161,7 @@
     <t>Id</t>
   </si>
   <si>
-    <t>27.05.2026 01:27:57 REPDOC</t>
+    <t>28.05.2026 01:19:38 REPDOC</t>
   </si>
   <si>
     <t/>
@@ -170,6 +170,69 @@
     <t>voller Satz</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>11,3</t>
+  </si>
+  <si>
+    <t>4100420097010</t>
+  </si>
+  <si>
+    <t>Falsch</t>
+  </si>
+  <si>
+    <t>Stck</t>
+  </si>
+  <si>
+    <t>{2E48AA74-C5AD-436B-B260-2BB350D8D8E6}</t>
+  </si>
+  <si>
+    <t>{00000000-0000-0000-0000-000000000000}</t>
+  </si>
+  <si>
+    <t>01-SELECT</t>
+  </si>
+  <si>
+    <t>Wahr</t>
+  </si>
+  <si>
+    <t>9701</t>
+  </si>
+  <si>
+    <t>LIQUI MOLY</t>
+  </si>
+  <si>
+    <t>44-Werkzeuge/Werkstattausrüstung</t>
+  </si>
+  <si>
+    <t>Motoröl Special Tec AA 0W-20 1L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                     9701</t>
+  </si>
+  <si>
+    <t>{B35FD5C0-C44B-4896-97A2-EC96057E7376}</t>
+  </si>
+  <si>
+    <t>50,16</t>
+  </si>
+  <si>
+    <t>4100420097348</t>
+  </si>
+  <si>
+    <t>9734</t>
+  </si>
+  <si>
+    <t>Motoröl Special Tec AA 0W-20 5L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                     9734</t>
+  </si>
+  <si>
+    <t>{FB5804C7-4B3E-4A3B-9B0E-8BBE04B6F4EB}</t>
+  </si>
+  <si>
     <t>48,16</t>
   </si>
   <si>
@@ -179,33 +242,12 @@
     <t>4025377215051</t>
   </si>
   <si>
-    <t>Falsch</t>
-  </si>
-  <si>
-    <t>Stck</t>
-  </si>
-  <si>
-    <t>{2E48AA74-C5AD-436B-B260-2BB350D8D8E6}</t>
-  </si>
-  <si>
-    <t>{00000000-0000-0000-0000-000000000000}</t>
-  </si>
-  <si>
-    <t>01-SELECT</t>
-  </si>
-  <si>
-    <t>Wahr</t>
-  </si>
-  <si>
     <t>215005</t>
   </si>
   <si>
     <t>EUROLUB</t>
   </si>
   <si>
-    <t>44-Werkzeuge/Werkstattausrüstung</t>
-  </si>
-  <si>
     <t>Motoröl 5L Longlife/Spezial 0W-20</t>
   </si>
   <si>
@@ -216,9 +258,6 @@
   </si>
   <si>
     <t>{222D56F3-EA0C-4493-889A-CD145C799928}</t>
-  </si>
-  <si>
-    <t>0</t>
   </si>
   <si>
     <t>42,64</t>
@@ -1608,7 +1647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AW44"/>
+  <dimension ref="A1:AW46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="0"/>
   <cols>
     <col min="3" max="3" width="16" customWidth="1"/>
@@ -1634,7 +1673,7 @@
     <col min="39" max="39" width="5" customWidth="1"/>
     <col min="40" max="40" width="7" customWidth="1"/>
     <col min="41" max="41" width="15" customWidth="1"/>
-    <col min="42" max="42" width="9" customWidth="1"/>
+    <col min="42" max="42" width="11" customWidth="1"/>
     <col min="43" max="43" width="33" customWidth="1"/>
     <col min="44" max="44" width="5" customWidth="1"/>
     <col min="45" max="45" width="41" customWidth="1"/>
@@ -1816,7 +1855,7 @@
         <v>50</v>
       </c>
       <c r="H2" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" s="6">
         <v>0</v>
@@ -1831,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N2" s="5" t="s">
         <v>56</v>
@@ -1852,9 +1891,6 @@
         <v>0</v>
       </c>
       <c r="T2" s="6">
-        <v>1</v>
-      </c>
-      <c r="U2" s="6">
         <v>0</v>
       </c>
       <c r="V2" t="s">
@@ -1882,7 +1918,7 @@
         <v>1</v>
       </c>
       <c r="AH2" s="6">
-        <v>93.89</v>
+        <v>19.49</v>
       </c>
       <c r="AI2" s="5" t="s">
         <v>50</v>
@@ -1891,7 +1927,7 @@
         <v>0</v>
       </c>
       <c r="AN2" s="6">
-        <v>78.9</v>
+        <v>16.38</v>
       </c>
       <c r="AO2" s="5" t="s">
         <v>61</v>
@@ -1909,16 +1945,16 @@
         <v>64</v>
       </c>
       <c r="AT2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AU2" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="AU2" s="5" t="s">
-        <v>66</v>
       </c>
       <c r="AV2" s="5" t="s">
         <v>61</v>
       </c>
       <c r="AW2" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" ht="15">
@@ -1932,22 +1968,22 @@
         <v>51</v>
       </c>
       <c r="E3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="6">
+        <v>0</v>
+      </c>
+      <c r="I3" s="6">
+        <v>0</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="F3" t="s">
-        <v>69</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H3" s="6">
-        <v>0</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="K3" t="s">
         <v>55</v>
@@ -1956,7 +1992,7 @@
         <v>0</v>
       </c>
       <c r="M3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N3" s="5" t="s">
         <v>56</v>
@@ -1979,9 +2015,6 @@
       <c r="T3" s="6">
         <v>0</v>
       </c>
-      <c r="U3" s="6">
-        <v>0</v>
-      </c>
       <c r="V3" t="s">
         <v>60</v>
       </c>
@@ -2007,7 +2040,7 @@
         <v>1</v>
       </c>
       <c r="AH3" s="6">
-        <v>148.75</v>
+        <v>86.49</v>
       </c>
       <c r="AI3" s="5" t="s">
         <v>50</v>
@@ -2016,10 +2049,10 @@
         <v>0</v>
       </c>
       <c r="AN3" s="6">
-        <v>125</v>
+        <v>72.68</v>
       </c>
       <c r="AO3" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="AP3" s="5" t="s">
         <v>62</v>
@@ -2031,19 +2064,19 @@
         <v>50</v>
       </c>
       <c r="AS3" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="AT3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AU3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="AV3" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="AW3" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="AT3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="AU3" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="AV3" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="AW3" s="9" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="4" ht="15">
@@ -2057,22 +2090,22 @@
         <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>50</v>
       </c>
       <c r="H4" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="6">
         <v>0</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="K4" t="s">
         <v>55</v>
@@ -2081,7 +2114,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>56</v>
@@ -2132,7 +2165,7 @@
         <v>1</v>
       </c>
       <c r="AH4" s="6">
-        <v>178.5</v>
+        <v>93.89</v>
       </c>
       <c r="AI4" s="5" t="s">
         <v>50</v>
@@ -2141,13 +2174,13 @@
         <v>0</v>
       </c>
       <c r="AN4" s="6">
-        <v>150</v>
+        <v>78.9</v>
       </c>
       <c r="AO4" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AP4" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ4" s="5" t="s">
         <v>63</v>
@@ -2156,19 +2189,19 @@
         <v>50</v>
       </c>
       <c r="AS4" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="AT4" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="AU4" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="AT4" s="5" t="s">
+      <c r="AV4" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AW4" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="AU4" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="AV4" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="AW4" s="9" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="5" ht="15">
@@ -2182,10 +2215,10 @@
         <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>50</v>
@@ -2197,7 +2230,7 @@
         <v>0</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="K5" t="s">
         <v>55</v>
@@ -2206,7 +2239,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>56</v>
@@ -2257,7 +2290,7 @@
         <v>1</v>
       </c>
       <c r="AH5" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI5" s="5" t="s">
         <v>50</v>
@@ -2266,13 +2299,13 @@
         <v>0</v>
       </c>
       <c r="AN5" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO5" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AP5" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ5" s="5" t="s">
         <v>63</v>
@@ -2281,19 +2314,19 @@
         <v>50</v>
       </c>
       <c r="AS5" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT5" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="AU5" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="AT5" s="5" t="s">
+      <c r="AV5" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AU5" s="5" t="s">
+      <c r="AW5" s="9" t="s">
         <v>89</v>
-      </c>
-      <c r="AV5" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW5" s="9" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="6" ht="15">
@@ -2307,10 +2340,10 @@
         <v>51</v>
       </c>
       <c r="E6" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>50</v>
@@ -2322,7 +2355,7 @@
         <v>0</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="K6" t="s">
         <v>55</v>
@@ -2331,7 +2364,7 @@
         <v>0</v>
       </c>
       <c r="M6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>56</v>
@@ -2343,7 +2376,7 @@
         <v>57</v>
       </c>
       <c r="Q6" s="9" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>59</v>
@@ -2352,7 +2385,7 @@
         <v>0</v>
       </c>
       <c r="T6" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" s="6">
         <v>0</v>
@@ -2382,7 +2415,7 @@
         <v>1</v>
       </c>
       <c r="AH6" s="6">
-        <v>148.75</v>
+        <v>178.5</v>
       </c>
       <c r="AI6" s="5" t="s">
         <v>50</v>
@@ -2391,13 +2424,13 @@
         <v>0</v>
       </c>
       <c r="AN6" s="6">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="AO6" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="AP6" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ6" s="5" t="s">
         <v>63</v>
@@ -2406,19 +2439,19 @@
         <v>50</v>
       </c>
       <c r="AS6" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="AT6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU6" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="AT6" s="5" t="s">
+      <c r="AV6" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="AU6" s="5" t="s">
+      <c r="AW6" s="9" t="s">
         <v>97</v>
-      </c>
-      <c r="AV6" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="AW6" s="9" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="7" ht="15">
@@ -2432,10 +2465,10 @@
         <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>50</v>
@@ -2447,7 +2480,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="K7" t="s">
         <v>55</v>
@@ -2456,7 +2489,7 @@
         <v>0</v>
       </c>
       <c r="M7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="N7" s="5" t="s">
         <v>56</v>
@@ -2519,10 +2552,10 @@
         <v>25</v>
       </c>
       <c r="AO7" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="AP7" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ7" s="5" t="s">
         <v>63</v>
@@ -2531,19 +2564,19 @@
         <v>50</v>
       </c>
       <c r="AS7" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AT7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="AU7" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="AV7" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AT7" s="5" t="s">
+      <c r="AW7" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="AU7" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="AV7" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="AW7" s="9" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="8" ht="15">
@@ -2557,10 +2590,10 @@
         <v>51</v>
       </c>
       <c r="E8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>50</v>
@@ -2569,7 +2602,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>50</v>
@@ -2581,7 +2614,7 @@
         <v>0</v>
       </c>
       <c r="M8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="N8" s="5" t="s">
         <v>56</v>
@@ -2593,7 +2626,7 @@
         <v>57</v>
       </c>
       <c r="Q8" s="9" t="s">
-        <v>58</v>
+        <v>106</v>
       </c>
       <c r="R8" s="5" t="s">
         <v>59</v>
@@ -2644,10 +2677,10 @@
         <v>125</v>
       </c>
       <c r="AO8" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="AP8" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ8" s="5" t="s">
         <v>63</v>
@@ -2656,19 +2689,19 @@
         <v>50</v>
       </c>
       <c r="AS8" s="5" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="AT8" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="AU8" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="AU8" s="5" t="s">
+      <c r="AV8" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="AV8" s="5" t="s">
+      <c r="AW8" s="9" t="s">
         <v>112</v>
-      </c>
-      <c r="AW8" s="9" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="9" ht="15">
@@ -2682,22 +2715,22 @@
         <v>51</v>
       </c>
       <c r="E9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" s="6">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="5" t="s">
         <v>114</v>
-      </c>
-      <c r="F9" t="s">
-        <v>114</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H9" s="6">
-        <v>0</v>
-      </c>
-      <c r="I9" s="6">
-        <v>4</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="K9" t="s">
         <v>55</v>
@@ -2706,7 +2739,7 @@
         <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="N9" s="5" t="s">
         <v>56</v>
@@ -2769,10 +2802,10 @@
         <v>25</v>
       </c>
       <c r="AO9" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AP9" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ9" s="5" t="s">
         <v>63</v>
@@ -2781,7 +2814,7 @@
         <v>50</v>
       </c>
       <c r="AS9" s="5" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="AT9" s="5" t="s">
         <v>117</v>
@@ -2819,10 +2852,10 @@
         <v>0</v>
       </c>
       <c r="I10" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>122</v>
+        <v>50</v>
       </c>
       <c r="K10" t="s">
         <v>55</v>
@@ -2843,7 +2876,7 @@
         <v>57</v>
       </c>
       <c r="Q10" s="9" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="R10" s="5" t="s">
         <v>59</v>
@@ -2882,7 +2915,7 @@
         <v>1</v>
       </c>
       <c r="AH10" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI10" s="5" t="s">
         <v>50</v>
@@ -2891,13 +2924,13 @@
         <v>0</v>
       </c>
       <c r="AN10" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO10" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AP10" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ10" s="5" t="s">
         <v>63</v>
@@ -2906,19 +2939,19 @@
         <v>50</v>
       </c>
       <c r="AS10" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="AT10" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AU10" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="AV10" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="AT10" s="5" t="s">
+      <c r="AW10" s="9" t="s">
         <v>126</v>
-      </c>
-      <c r="AU10" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="AV10" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="AW10" s="9" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="11" ht="15">
@@ -2932,10 +2965,10 @@
         <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F11" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>50</v>
@@ -2944,10 +2977,10 @@
         <v>0</v>
       </c>
       <c r="I11" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K11" t="s">
         <v>55</v>
@@ -2956,7 +2989,7 @@
         <v>0</v>
       </c>
       <c r="M11" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="N11" s="5" t="s">
         <v>56</v>
@@ -2968,7 +3001,7 @@
         <v>57</v>
       </c>
       <c r="Q11" s="9" t="s">
-        <v>132</v>
+        <v>58</v>
       </c>
       <c r="R11" s="5" t="s">
         <v>59</v>
@@ -3007,7 +3040,7 @@
         <v>1</v>
       </c>
       <c r="AH11" s="6">
-        <v>148.75</v>
+        <v>29.75</v>
       </c>
       <c r="AI11" s="5" t="s">
         <v>50</v>
@@ -3016,13 +3049,13 @@
         <v>0</v>
       </c>
       <c r="AN11" s="6">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AO11" s="5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="AP11" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ11" s="5" t="s">
         <v>63</v>
@@ -3031,19 +3064,19 @@
         <v>50</v>
       </c>
       <c r="AS11" s="5" t="s">
-        <v>72</v>
+        <v>116</v>
       </c>
       <c r="AT11" s="5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="AU11" s="5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="AV11" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="AW11" s="9" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" ht="15">
@@ -3057,10 +3090,10 @@
         <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>134</v>
       </c>
       <c r="F12" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>50</v>
@@ -3072,7 +3105,7 @@
         <v>0</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="K12" t="s">
         <v>55</v>
@@ -3081,7 +3114,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="N12" s="5" t="s">
         <v>56</v>
@@ -3093,7 +3126,7 @@
         <v>57</v>
       </c>
       <c r="Q12" s="9" t="s">
-        <v>58</v>
+        <v>136</v>
       </c>
       <c r="R12" s="5" t="s">
         <v>59</v>
@@ -3132,7 +3165,7 @@
         <v>1</v>
       </c>
       <c r="AH12" s="6">
-        <v>148.75</v>
+        <v>29.75</v>
       </c>
       <c r="AI12" s="5" t="s">
         <v>50</v>
@@ -3141,13 +3174,13 @@
         <v>0</v>
       </c>
       <c r="AN12" s="6">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AO12" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="AP12" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ12" s="5" t="s">
         <v>63</v>
@@ -3156,19 +3189,19 @@
         <v>50</v>
       </c>
       <c r="AS12" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="AT12" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="AU12" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="AV12" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="AT12" s="5" t="s">
+      <c r="AW12" s="9" t="s">
         <v>142</v>
-      </c>
-      <c r="AU12" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="AV12" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="AW12" s="9" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="13" ht="15">
@@ -3182,10 +3215,10 @@
         <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F13" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>50</v>
@@ -3194,10 +3227,10 @@
         <v>0</v>
       </c>
       <c r="I13" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="K13" t="s">
         <v>55</v>
@@ -3206,7 +3239,7 @@
         <v>0</v>
       </c>
       <c r="M13" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="N13" s="5" t="s">
         <v>56</v>
@@ -3218,7 +3251,7 @@
         <v>57</v>
       </c>
       <c r="Q13" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="R13" s="5" t="s">
         <v>59</v>
@@ -3257,7 +3290,7 @@
         <v>1</v>
       </c>
       <c r="AH13" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI13" s="5" t="s">
         <v>50</v>
@@ -3266,13 +3299,13 @@
         <v>0</v>
       </c>
       <c r="AN13" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO13" s="5" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="AP13" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ13" s="5" t="s">
         <v>63</v>
@@ -3281,19 +3314,19 @@
         <v>50</v>
       </c>
       <c r="AS13" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="AT13" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="AU13" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="AV13" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="AW13" s="9" t="s">
         <v>150</v>
-      </c>
-      <c r="AT13" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="AU13" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="AV13" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="AW13" s="9" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="14" ht="15">
@@ -3307,10 +3340,10 @@
         <v>51</v>
       </c>
       <c r="E14" t="s">
-        <v>155</v>
+        <v>52</v>
       </c>
       <c r="F14" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>50</v>
@@ -3322,7 +3355,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="K14" t="s">
         <v>55</v>
@@ -3331,7 +3364,7 @@
         <v>0</v>
       </c>
       <c r="M14" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="N14" s="5" t="s">
         <v>56</v>
@@ -3343,7 +3376,7 @@
         <v>57</v>
       </c>
       <c r="Q14" s="9" t="s">
-        <v>148</v>
+        <v>58</v>
       </c>
       <c r="R14" s="5" t="s">
         <v>59</v>
@@ -3394,10 +3427,10 @@
         <v>125</v>
       </c>
       <c r="AO14" s="5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="AP14" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ14" s="5" t="s">
         <v>63</v>
@@ -3406,19 +3439,19 @@
         <v>50</v>
       </c>
       <c r="AS14" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="AT14" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="AU14" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="AV14" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="AW14" s="9" t="s">
         <v>158</v>
-      </c>
-      <c r="AT14" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="AU14" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="AV14" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="AW14" s="9" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="15" ht="15">
@@ -3432,10 +3465,10 @@
         <v>51</v>
       </c>
       <c r="E15" t="s">
-        <v>68</v>
+        <v>159</v>
       </c>
       <c r="F15" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>50</v>
@@ -3447,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="K15" t="s">
         <v>55</v>
@@ -3456,10 +3489,10 @@
         <v>0</v>
       </c>
       <c r="M15" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>164</v>
+        <v>56</v>
       </c>
       <c r="O15" s="6">
         <v>0</v>
@@ -3468,7 +3501,7 @@
         <v>57</v>
       </c>
       <c r="Q15" s="9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="R15" s="5" t="s">
         <v>59</v>
@@ -3476,11 +3509,14 @@
       <c r="S15" s="6">
         <v>0</v>
       </c>
+      <c r="T15" s="6">
+        <v>0</v>
+      </c>
       <c r="U15" s="6">
         <v>0</v>
       </c>
       <c r="V15" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="W15" s="6">
         <v>0</v>
@@ -3504,40 +3540,43 @@
         <v>1</v>
       </c>
       <c r="AH15" s="6">
-        <v>20.83</v>
+        <v>29.75</v>
       </c>
       <c r="AI15" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="AM15" s="6">
+        <v>0</v>
+      </c>
       <c r="AN15" s="6">
-        <v>17.5</v>
+        <v>25</v>
       </c>
       <c r="AO15" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="AP15" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ15" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS15" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="AT15" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="AU15" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="AV15" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="AP15" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AQ15" s="5" t="s">
+      <c r="AW15" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="AR15" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS15" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="AT15" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="AU15" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="AV15" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="AW15" s="9" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="16" ht="15">
@@ -3551,10 +3590,10 @@
         <v>51</v>
       </c>
       <c r="E16" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="F16" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>50</v>
@@ -3566,7 +3605,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="K16" t="s">
         <v>55</v>
@@ -3575,7 +3614,7 @@
         <v>0</v>
       </c>
       <c r="M16" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="N16" s="5" t="s">
         <v>56</v>
@@ -3587,7 +3626,7 @@
         <v>57</v>
       </c>
       <c r="Q16" s="9" t="s">
-        <v>58</v>
+        <v>161</v>
       </c>
       <c r="R16" s="5" t="s">
         <v>59</v>
@@ -3626,7 +3665,7 @@
         <v>1</v>
       </c>
       <c r="AH16" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI16" s="5" t="s">
         <v>50</v>
@@ -3635,13 +3674,13 @@
         <v>0</v>
       </c>
       <c r="AN16" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO16" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="AP16" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ16" s="5" t="s">
         <v>63</v>
@@ -3650,19 +3689,19 @@
         <v>50</v>
       </c>
       <c r="AS16" s="5" t="s">
-        <v>87</v>
+        <v>171</v>
       </c>
       <c r="AT16" s="5" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="AU16" s="5" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="AV16" s="5" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AW16" s="9" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" ht="15">
@@ -3676,10 +3715,10 @@
         <v>51</v>
       </c>
       <c r="E17" t="s">
-        <v>180</v>
+        <v>52</v>
       </c>
       <c r="F17" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>50</v>
@@ -3691,7 +3730,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>181</v>
+        <v>50</v>
       </c>
       <c r="K17" t="s">
         <v>55</v>
@@ -3700,10 +3739,10 @@
         <v>0</v>
       </c>
       <c r="M17" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>56</v>
+        <v>177</v>
       </c>
       <c r="O17" s="6">
         <v>0</v>
@@ -3712,7 +3751,7 @@
         <v>57</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>58</v>
+        <v>178</v>
       </c>
       <c r="R17" s="5" t="s">
         <v>59</v>
@@ -3720,14 +3759,11 @@
       <c r="S17" s="6">
         <v>0</v>
       </c>
-      <c r="T17" s="6">
-        <v>0</v>
-      </c>
       <c r="U17" s="6">
         <v>0</v>
       </c>
       <c r="V17" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="W17" s="6">
         <v>0</v>
@@ -3751,43 +3787,40 @@
         <v>1</v>
       </c>
       <c r="AH17" s="6">
-        <v>148.75</v>
+        <v>20.83</v>
       </c>
       <c r="AI17" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AM17" s="6">
-        <v>0</v>
-      </c>
       <c r="AN17" s="6">
-        <v>125</v>
+        <v>17.5</v>
       </c>
       <c r="AO17" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="AP17" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ17" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR17" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS17" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="AT17" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="AP17" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AQ17" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AR17" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS17" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="AT17" s="5" t="s">
+      <c r="AU17" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="AU17" s="5" t="s">
+      <c r="AV17" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="AV17" s="5" t="s">
+      <c r="AW17" s="9" t="s">
         <v>185</v>
-      </c>
-      <c r="AW17" s="9" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="18" ht="15">
@@ -3801,22 +3834,22 @@
         <v>51</v>
       </c>
       <c r="E18" t="s">
+        <v>186</v>
+      </c>
+      <c r="F18" t="s">
+        <v>186</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" s="6">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5" t="s">
         <v>187</v>
-      </c>
-      <c r="F18" t="s">
-        <v>187</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H18" s="6">
-        <v>0</v>
-      </c>
-      <c r="I18" s="6">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>188</v>
       </c>
       <c r="K18" t="s">
         <v>55</v>
@@ -3825,7 +3858,7 @@
         <v>0</v>
       </c>
       <c r="M18" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N18" s="5" t="s">
         <v>56</v>
@@ -3876,7 +3909,7 @@
         <v>1</v>
       </c>
       <c r="AH18" s="6">
-        <v>104.13</v>
+        <v>29.75</v>
       </c>
       <c r="AI18" s="5" t="s">
         <v>50</v>
@@ -3885,13 +3918,13 @@
         <v>0</v>
       </c>
       <c r="AN18" s="6">
-        <v>87.5</v>
+        <v>25</v>
       </c>
       <c r="AO18" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AP18" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ18" s="5" t="s">
         <v>63</v>
@@ -3900,19 +3933,19 @@
         <v>50</v>
       </c>
       <c r="AS18" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AT18" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="AU18" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="AT18" s="5" t="s">
+      <c r="AV18" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="AU18" s="5" t="s">
+      <c r="AW18" s="9" t="s">
         <v>192</v>
-      </c>
-      <c r="AV18" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="AW18" s="9" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="19" ht="15">
@@ -3926,10 +3959,10 @@
         <v>51</v>
       </c>
       <c r="E19" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F19" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>50</v>
@@ -3938,10 +3971,10 @@
         <v>0</v>
       </c>
       <c r="I19" s="6">
-        <v>6.75</v>
+        <v>0</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>50</v>
+        <v>194</v>
       </c>
       <c r="K19" t="s">
         <v>55</v>
@@ -3950,10 +3983,10 @@
         <v>0</v>
       </c>
       <c r="M19" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>164</v>
+        <v>56</v>
       </c>
       <c r="O19" s="6">
         <v>0</v>
@@ -3962,7 +3995,7 @@
         <v>57</v>
       </c>
       <c r="Q19" s="9" t="s">
-        <v>196</v>
+        <v>58</v>
       </c>
       <c r="R19" s="5" t="s">
         <v>59</v>
@@ -3971,7 +4004,10 @@
         <v>0</v>
       </c>
       <c r="T19" s="6">
-        <v>197.05</v>
+        <v>0</v>
+      </c>
+      <c r="U19" s="6">
+        <v>0</v>
       </c>
       <c r="V19" t="s">
         <v>60</v>
@@ -3998,40 +4034,43 @@
         <v>1</v>
       </c>
       <c r="AH19" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI19" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="AM19" s="6">
+        <v>0</v>
+      </c>
       <c r="AN19" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO19" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="AP19" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ19" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR19" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS19" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="AT19" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="AU19" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="AP19" s="5" t="s">
+      <c r="AV19" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="AQ19" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR19" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS19" s="5" t="s">
+      <c r="AW19" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="AT19" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="AU19" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV19" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="AW19" s="9" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="20" ht="15">
@@ -4045,10 +4084,10 @@
         <v>51</v>
       </c>
       <c r="E20" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="F20" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>50</v>
@@ -4060,7 +4099,7 @@
         <v>0</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="K20" t="s">
         <v>55</v>
@@ -4069,7 +4108,7 @@
         <v>0</v>
       </c>
       <c r="M20" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="N20" s="5" t="s">
         <v>56</v>
@@ -4120,7 +4159,7 @@
         <v>1</v>
       </c>
       <c r="AH20" s="6">
-        <v>148.75</v>
+        <v>104.13</v>
       </c>
       <c r="AI20" s="5" t="s">
         <v>50</v>
@@ -4129,13 +4168,13 @@
         <v>0</v>
       </c>
       <c r="AN20" s="6">
-        <v>125</v>
+        <v>87.5</v>
       </c>
       <c r="AO20" s="5" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="AP20" s="5" t="s">
-        <v>207</v>
+        <v>77</v>
       </c>
       <c r="AQ20" s="5" t="s">
         <v>63</v>
@@ -4144,19 +4183,19 @@
         <v>50</v>
       </c>
       <c r="AS20" s="5" t="s">
-        <v>72</v>
+        <v>203</v>
       </c>
       <c r="AT20" s="5" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="AU20" s="5" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="AV20" s="5" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="AW20" s="9" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" ht="15">
@@ -4170,10 +4209,10 @@
         <v>51</v>
       </c>
       <c r="E21" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F21" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>50</v>
@@ -4182,10 +4221,10 @@
         <v>0</v>
       </c>
       <c r="I21" s="6">
-        <v>0</v>
+        <v>6.75</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>213</v>
+        <v>50</v>
       </c>
       <c r="K21" t="s">
         <v>55</v>
@@ -4194,10 +4233,10 @@
         <v>0</v>
       </c>
       <c r="M21" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="N21" s="5" t="s">
-        <v>56</v>
+        <v>177</v>
       </c>
       <c r="O21" s="6">
         <v>0</v>
@@ -4206,7 +4245,7 @@
         <v>57</v>
       </c>
       <c r="Q21" s="9" t="s">
-        <v>132</v>
+        <v>209</v>
       </c>
       <c r="R21" s="5" t="s">
         <v>59</v>
@@ -4215,10 +4254,7 @@
         <v>0</v>
       </c>
       <c r="T21" s="6">
-        <v>0</v>
-      </c>
-      <c r="U21" s="6">
-        <v>0</v>
+        <v>197.05</v>
       </c>
       <c r="V21" t="s">
         <v>60</v>
@@ -4245,43 +4281,40 @@
         <v>1</v>
       </c>
       <c r="AH21" s="6">
-        <v>148.75</v>
+        <v>29.75</v>
       </c>
       <c r="AI21" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AM21" s="6">
-        <v>0</v>
-      </c>
       <c r="AN21" s="6">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AO21" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="AP21" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="AQ21" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS21" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="AT21" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="AU21" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="AP21" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="AQ21" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AR21" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS21" s="5" t="s">
+      <c r="AV21" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="AT21" s="5" t="s">
+      <c r="AW21" s="9" t="s">
         <v>216</v>
-      </c>
-      <c r="AU21" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="AV21" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="AW21" s="9" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="22" ht="15">
@@ -4295,10 +4328,10 @@
         <v>51</v>
       </c>
       <c r="E22" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F22" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>50</v>
@@ -4310,7 +4343,7 @@
         <v>0</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="K22" t="s">
         <v>55</v>
@@ -4319,7 +4352,7 @@
         <v>0</v>
       </c>
       <c r="M22" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="N22" s="5" t="s">
         <v>56</v>
@@ -4331,7 +4364,7 @@
         <v>57</v>
       </c>
       <c r="Q22" s="9" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="R22" s="5" t="s">
         <v>59</v>
@@ -4370,7 +4403,7 @@
         <v>1</v>
       </c>
       <c r="AH22" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI22" s="5" t="s">
         <v>50</v>
@@ -4379,13 +4412,13 @@
         <v>0</v>
       </c>
       <c r="AN22" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO22" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="AP22" s="5" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="AQ22" s="5" t="s">
         <v>63</v>
@@ -4394,19 +4427,19 @@
         <v>50</v>
       </c>
       <c r="AS22" s="5" t="s">
-        <v>125</v>
+        <v>85</v>
       </c>
       <c r="AT22" s="5" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="AU22" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="AV22" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="AV22" s="5" t="s">
+      <c r="AW22" s="9" t="s">
         <v>224</v>
-      </c>
-      <c r="AW22" s="9" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="23" ht="15">
@@ -4420,22 +4453,22 @@
         <v>51</v>
       </c>
       <c r="E23" t="s">
-        <v>68</v>
+        <v>225</v>
       </c>
       <c r="F23" t="s">
+        <v>225</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H23" s="6">
+        <v>0</v>
+      </c>
+      <c r="I23" s="6">
+        <v>0</v>
+      </c>
+      <c r="J23" s="5" t="s">
         <v>226</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H23" s="6">
-        <v>0</v>
-      </c>
-      <c r="I23" s="6">
-        <v>0</v>
-      </c>
-      <c r="J23" s="5" t="s">
-        <v>227</v>
       </c>
       <c r="K23" t="s">
         <v>55</v>
@@ -4444,7 +4477,7 @@
         <v>0</v>
       </c>
       <c r="M23" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="N23" s="5" t="s">
         <v>56</v>
@@ -4456,7 +4489,7 @@
         <v>57</v>
       </c>
       <c r="Q23" s="9" t="s">
-        <v>58</v>
+        <v>145</v>
       </c>
       <c r="R23" s="5" t="s">
         <v>59</v>
@@ -4507,10 +4540,10 @@
         <v>125</v>
       </c>
       <c r="AO23" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AP23" s="5" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="AQ23" s="5" t="s">
         <v>63</v>
@@ -4519,7 +4552,7 @@
         <v>50</v>
       </c>
       <c r="AS23" s="5" t="s">
-        <v>72</v>
+        <v>228</v>
       </c>
       <c r="AT23" s="5" t="s">
         <v>229</v>
@@ -4545,7 +4578,7 @@
         <v>51</v>
       </c>
       <c r="E24" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="F24" t="s">
         <v>233</v>
@@ -4581,7 +4614,7 @@
         <v>57</v>
       </c>
       <c r="Q24" s="9" t="s">
-        <v>58</v>
+        <v>136</v>
       </c>
       <c r="R24" s="5" t="s">
         <v>59</v>
@@ -4635,7 +4668,7 @@
         <v>235</v>
       </c>
       <c r="AP24" s="5" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="AQ24" s="5" t="s">
         <v>63</v>
@@ -4644,19 +4677,19 @@
         <v>50</v>
       </c>
       <c r="AS24" s="5" t="s">
-        <v>236</v>
+        <v>138</v>
       </c>
       <c r="AT24" s="5" t="s">
         <v>229</v>
       </c>
       <c r="AU24" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="AV24" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="AV24" s="5" t="s">
+      <c r="AW24" s="9" t="s">
         <v>238</v>
-      </c>
-      <c r="AW24" s="9" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="25" ht="15">
@@ -4670,22 +4703,22 @@
         <v>51</v>
       </c>
       <c r="E25" t="s">
+        <v>52</v>
+      </c>
+      <c r="F25" t="s">
+        <v>239</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H25" s="6">
+        <v>0</v>
+      </c>
+      <c r="I25" s="6">
+        <v>0</v>
+      </c>
+      <c r="J25" s="5" t="s">
         <v>240</v>
-      </c>
-      <c r="F25" t="s">
-        <v>241</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H25" s="6">
-        <v>0</v>
-      </c>
-      <c r="I25" s="6">
-        <v>8.3</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>242</v>
       </c>
       <c r="K25" t="s">
         <v>55</v>
@@ -4694,10 +4727,10 @@
         <v>0</v>
       </c>
       <c r="M25" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="N25" s="5" t="s">
-        <v>164</v>
+        <v>56</v>
       </c>
       <c r="O25" s="6">
         <v>0</v>
@@ -4706,7 +4739,7 @@
         <v>57</v>
       </c>
       <c r="Q25" s="9" t="s">
-        <v>244</v>
+        <v>58</v>
       </c>
       <c r="R25" s="5" t="s">
         <v>59</v>
@@ -4715,7 +4748,7 @@
         <v>0</v>
       </c>
       <c r="T25" s="6">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="U25" s="6">
         <v>0</v>
@@ -4745,7 +4778,7 @@
         <v>1</v>
       </c>
       <c r="AH25" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI25" s="5" t="s">
         <v>50</v>
@@ -4754,13 +4787,13 @@
         <v>0</v>
       </c>
       <c r="AN25" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO25" s="5" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="AP25" s="5" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="AQ25" s="5" t="s">
         <v>63</v>
@@ -4769,19 +4802,19 @@
         <v>50</v>
       </c>
       <c r="AS25" s="5" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="AT25" s="5" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="AU25" s="5" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="AV25" s="5" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="AW25" s="9" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26" ht="15">
@@ -4795,10 +4828,10 @@
         <v>51</v>
       </c>
       <c r="E26" t="s">
-        <v>212</v>
+        <v>52</v>
       </c>
       <c r="F26" t="s">
-        <v>212</v>
+        <v>246</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>50</v>
@@ -4810,16 +4843,16 @@
         <v>0</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>50</v>
+        <v>247</v>
       </c>
       <c r="K26" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="L26" s="7">
         <v>0</v>
       </c>
       <c r="M26" t="s">
-        <v>212</v>
+        <v>246</v>
       </c>
       <c r="N26" s="5" t="s">
         <v>56</v>
@@ -4831,7 +4864,7 @@
         <v>57</v>
       </c>
       <c r="Q26" s="9" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="R26" s="5" t="s">
         <v>59</v>
@@ -4839,8 +4872,14 @@
       <c r="S26" s="6">
         <v>0</v>
       </c>
+      <c r="T26" s="6">
+        <v>0</v>
+      </c>
+      <c r="U26" s="6">
+        <v>0</v>
+      </c>
       <c r="V26" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="W26" s="6">
         <v>0</v>
@@ -4864,40 +4903,43 @@
         <v>1</v>
       </c>
       <c r="AH26" s="6">
-        <v>148.75</v>
+        <v>29.75</v>
       </c>
       <c r="AI26" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="AM26" s="6">
+        <v>0</v>
+      </c>
       <c r="AN26" s="6">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AO26" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="AP26" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="AQ26" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR26" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS26" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="AT26" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="AU26" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="AP26" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="AQ26" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR26" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS26" s="5" t="s">
+      <c r="AV26" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="AT26" s="5" t="s">
+      <c r="AW26" s="9" t="s">
         <v>252</v>
-      </c>
-      <c r="AU26" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="AV26" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="AW26" s="9" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="27" ht="15">
@@ -4911,10 +4953,10 @@
         <v>51</v>
       </c>
       <c r="E27" t="s">
-        <v>68</v>
+        <v>253</v>
       </c>
       <c r="F27" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>50</v>
@@ -4923,10 +4965,10 @@
         <v>0</v>
       </c>
       <c r="I27" s="6">
-        <v>0</v>
+        <v>8.3</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="K27" t="s">
         <v>55</v>
@@ -4938,7 +4980,7 @@
         <v>256</v>
       </c>
       <c r="N27" s="5" t="s">
-        <v>56</v>
+        <v>177</v>
       </c>
       <c r="O27" s="6">
         <v>0</v>
@@ -4947,7 +4989,7 @@
         <v>57</v>
       </c>
       <c r="Q27" s="9" t="s">
-        <v>58</v>
+        <v>257</v>
       </c>
       <c r="R27" s="5" t="s">
         <v>59</v>
@@ -4956,7 +4998,7 @@
         <v>0</v>
       </c>
       <c r="T27" s="6">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="U27" s="6">
         <v>0</v>
@@ -4986,7 +5028,7 @@
         <v>1</v>
       </c>
       <c r="AH27" s="6">
-        <v>41.65</v>
+        <v>29.75</v>
       </c>
       <c r="AI27" s="5" t="s">
         <v>50</v>
@@ -4995,13 +5037,13 @@
         <v>0</v>
       </c>
       <c r="AN27" s="6">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AO27" s="5" t="s">
         <v>258</v>
       </c>
       <c r="AP27" s="5" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="AQ27" s="5" t="s">
         <v>63</v>
@@ -5010,19 +5052,19 @@
         <v>50</v>
       </c>
       <c r="AS27" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="AT27" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="AT27" s="5" t="s">
+      <c r="AU27" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="AU27" s="5" t="s">
+      <c r="AV27" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="AV27" s="5" t="s">
+      <c r="AW27" s="9" t="s">
         <v>262</v>
-      </c>
-      <c r="AW27" s="9" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="28" ht="15">
@@ -5036,10 +5078,10 @@
         <v>51</v>
       </c>
       <c r="E28" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="F28" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>50</v>
@@ -5054,13 +5096,13 @@
         <v>50</v>
       </c>
       <c r="K28" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="L28" s="7">
         <v>0</v>
       </c>
       <c r="M28" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="N28" s="5" t="s">
         <v>56</v>
@@ -5072,7 +5114,7 @@
         <v>57</v>
       </c>
       <c r="Q28" s="9" t="s">
-        <v>58</v>
+        <v>106</v>
       </c>
       <c r="R28" s="5" t="s">
         <v>59</v>
@@ -5080,14 +5122,8 @@
       <c r="S28" s="6">
         <v>0</v>
       </c>
-      <c r="T28" s="6">
-        <v>0</v>
-      </c>
-      <c r="U28" s="6">
-        <v>0</v>
-      </c>
       <c r="V28" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="W28" s="6">
         <v>0</v>
@@ -5111,43 +5147,40 @@
         <v>1</v>
       </c>
       <c r="AH28" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI28" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AM28" s="6">
-        <v>0</v>
-      </c>
       <c r="AN28" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO28" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="AP28" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="AQ28" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR28" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS28" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="AP28" s="5" t="s">
+      <c r="AT28" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="AQ28" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR28" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS28" s="5" t="s">
+      <c r="AU28" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="AT28" s="5" t="s">
+      <c r="AV28" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="AU28" s="5" t="s">
+      <c r="AW28" s="9" t="s">
         <v>268</v>
-      </c>
-      <c r="AV28" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="AW28" s="9" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="29" ht="15">
@@ -5161,10 +5194,10 @@
         <v>51</v>
       </c>
       <c r="E29" t="s">
-        <v>271</v>
+        <v>52</v>
       </c>
       <c r="F29" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>50</v>
@@ -5176,7 +5209,7 @@
         <v>0</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="K29" t="s">
         <v>55</v>
@@ -5185,7 +5218,7 @@
         <v>0</v>
       </c>
       <c r="M29" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="N29" s="5" t="s">
         <v>56</v>
@@ -5236,7 +5269,7 @@
         <v>1</v>
       </c>
       <c r="AH29" s="6">
-        <v>29.75</v>
+        <v>41.65</v>
       </c>
       <c r="AI29" s="5" t="s">
         <v>50</v>
@@ -5245,13 +5278,13 @@
         <v>0</v>
       </c>
       <c r="AN29" s="6">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="AO29" s="5" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="AP29" s="5" t="s">
-        <v>265</v>
+        <v>220</v>
       </c>
       <c r="AQ29" s="5" t="s">
         <v>63</v>
@@ -5260,19 +5293,19 @@
         <v>50</v>
       </c>
       <c r="AS29" s="5" t="s">
-        <v>87</v>
+        <v>272</v>
       </c>
       <c r="AT29" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="AU29" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="AV29" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="AU29" s="5" t="s">
+      <c r="AW29" s="9" t="s">
         <v>276</v>
-      </c>
-      <c r="AV29" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="AW29" s="9" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="30" ht="15">
@@ -5286,10 +5319,10 @@
         <v>51</v>
       </c>
       <c r="E30" t="s">
-        <v>279</v>
+        <v>186</v>
       </c>
       <c r="F30" t="s">
-        <v>280</v>
+        <v>186</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>50</v>
@@ -5301,7 +5334,7 @@
         <v>0</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>281</v>
+        <v>50</v>
       </c>
       <c r="K30" t="s">
         <v>55</v>
@@ -5310,7 +5343,7 @@
         <v>0</v>
       </c>
       <c r="M30" t="s">
-        <v>279</v>
+        <v>186</v>
       </c>
       <c r="N30" s="5" t="s">
         <v>56</v>
@@ -5361,7 +5394,7 @@
         <v>1</v>
       </c>
       <c r="AH30" s="6">
-        <v>148.75</v>
+        <v>29.75</v>
       </c>
       <c r="AI30" s="5" t="s">
         <v>50</v>
@@ -5370,34 +5403,34 @@
         <v>0</v>
       </c>
       <c r="AN30" s="6">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AO30" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="AP30" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AQ30" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR30" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS30" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="AT30" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="AU30" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="AV30" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="AP30" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="AQ30" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AR30" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS30" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="AT30" s="5" t="s">
+      <c r="AW30" s="9" t="s">
         <v>283</v>
-      </c>
-      <c r="AU30" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="AV30" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="AW30" s="9" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="31" ht="15">
@@ -5411,10 +5444,10 @@
         <v>51</v>
       </c>
       <c r="E31" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F31" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>50</v>
@@ -5426,7 +5459,7 @@
         <v>0</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="K31" t="s">
         <v>55</v>
@@ -5435,7 +5468,7 @@
         <v>0</v>
       </c>
       <c r="M31" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="N31" s="5" t="s">
         <v>56</v>
@@ -5486,7 +5519,7 @@
         <v>1</v>
       </c>
       <c r="AH31" s="6">
-        <v>148.75</v>
+        <v>29.75</v>
       </c>
       <c r="AI31" s="5" t="s">
         <v>50</v>
@@ -5495,13 +5528,13 @@
         <v>0</v>
       </c>
       <c r="AN31" s="6">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AO31" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="AP31" s="5" t="s">
-        <v>207</v>
+        <v>278</v>
       </c>
       <c r="AQ31" s="5" t="s">
         <v>63</v>
@@ -5510,16 +5543,16 @@
         <v>50</v>
       </c>
       <c r="AS31" s="5" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="AT31" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="AU31" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="AV31" s="5" t="s">
         <v>290</v>
-      </c>
-      <c r="AU31" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="AV31" s="5" t="s">
-        <v>285</v>
       </c>
       <c r="AW31" s="9" t="s">
         <v>291</v>
@@ -5539,7 +5572,7 @@
         <v>292</v>
       </c>
       <c r="F32" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>50</v>
@@ -5551,7 +5584,7 @@
         <v>0</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K32" t="s">
         <v>55</v>
@@ -5611,7 +5644,7 @@
         <v>1</v>
       </c>
       <c r="AH32" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI32" s="5" t="s">
         <v>50</v>
@@ -5620,13 +5653,13 @@
         <v>0</v>
       </c>
       <c r="AN32" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO32" s="5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AP32" s="5" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="AQ32" s="5" t="s">
         <v>63</v>
@@ -5635,19 +5668,19 @@
         <v>50</v>
       </c>
       <c r="AS32" s="5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="AT32" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="AU32" s="5" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="AV32" s="5" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="AW32" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="33" ht="15">
@@ -5661,10 +5694,10 @@
         <v>51</v>
       </c>
       <c r="E33" t="s">
-        <v>68</v>
+        <v>300</v>
       </c>
       <c r="F33" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>50</v>
@@ -5676,7 +5709,7 @@
         <v>0</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K33" t="s">
         <v>55</v>
@@ -5685,7 +5718,7 @@
         <v>0</v>
       </c>
       <c r="M33" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="N33" s="5" t="s">
         <v>56</v>
@@ -5736,7 +5769,7 @@
         <v>1</v>
       </c>
       <c r="AH33" s="6">
-        <v>208.25</v>
+        <v>148.75</v>
       </c>
       <c r="AI33" s="5" t="s">
         <v>50</v>
@@ -5745,13 +5778,13 @@
         <v>0</v>
       </c>
       <c r="AN33" s="6">
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="AO33" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AP33" s="5" t="s">
-        <v>265</v>
+        <v>220</v>
       </c>
       <c r="AQ33" s="5" t="s">
         <v>63</v>
@@ -5760,19 +5793,19 @@
         <v>50</v>
       </c>
       <c r="AS33" s="5" t="s">
-        <v>302</v>
+        <v>85</v>
       </c>
       <c r="AT33" s="5" t="s">
         <v>303</v>
       </c>
       <c r="AU33" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="AV33" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="AW33" s="9" t="s">
         <v>304</v>
-      </c>
-      <c r="AV33" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="AW33" s="9" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="34" ht="15">
@@ -5786,10 +5819,10 @@
         <v>51</v>
       </c>
       <c r="E34" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="F34" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>50</v>
@@ -5801,7 +5834,7 @@
         <v>0</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>50</v>
+        <v>306</v>
       </c>
       <c r="K34" t="s">
         <v>55</v>
@@ -5810,10 +5843,10 @@
         <v>0</v>
       </c>
       <c r="M34" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="N34" s="5" t="s">
-        <v>164</v>
+        <v>56</v>
       </c>
       <c r="O34" s="6">
         <v>0</v>
@@ -5822,7 +5855,7 @@
         <v>57</v>
       </c>
       <c r="Q34" s="9" t="s">
-        <v>244</v>
+        <v>58</v>
       </c>
       <c r="R34" s="5" t="s">
         <v>59</v>
@@ -5831,7 +5864,7 @@
         <v>0</v>
       </c>
       <c r="T34" s="6">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="U34" s="6">
         <v>0</v>
@@ -5861,40 +5894,43 @@
         <v>1</v>
       </c>
       <c r="AH34" s="6">
-        <v>41.65</v>
+        <v>29.75</v>
       </c>
       <c r="AI34" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="AM34" s="6">
+        <v>0</v>
+      </c>
       <c r="AN34" s="6">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AO34" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="AP34" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AQ34" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR34" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS34" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="AT34" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="AU34" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="AP34" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="AQ34" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR34" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS34" s="5" t="s">
+      <c r="AV34" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="AT34" s="5" t="s">
+      <c r="AW34" s="9" t="s">
         <v>311</v>
-      </c>
-      <c r="AU34" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="AV34" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="AW34" s="9" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="35" ht="15">
@@ -5908,10 +5944,10 @@
         <v>51</v>
       </c>
       <c r="E35" t="s">
-        <v>315</v>
+        <v>52</v>
       </c>
       <c r="F35" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>50</v>
@@ -5923,7 +5959,7 @@
         <v>0</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>50</v>
+        <v>313</v>
       </c>
       <c r="K35" t="s">
         <v>55</v>
@@ -5932,7 +5968,7 @@
         <v>0</v>
       </c>
       <c r="M35" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="N35" s="5" t="s">
         <v>56</v>
@@ -5983,40 +6019,43 @@
         <v>1</v>
       </c>
       <c r="AH35" s="6">
-        <v>29.75</v>
+        <v>208.25</v>
       </c>
       <c r="AI35" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="AM35" s="6">
+        <v>0</v>
+      </c>
       <c r="AN35" s="6">
-        <v>25</v>
+        <v>175</v>
       </c>
       <c r="AO35" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="AP35" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AQ35" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR35" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS35" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="AT35" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="AU35" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="AP35" s="5" t="s">
+      <c r="AV35" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="AQ35" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR35" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS35" s="5" t="s">
+      <c r="AW35" s="9" t="s">
         <v>319</v>
-      </c>
-      <c r="AT35" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="AU35" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="AV35" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="AW35" s="9" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="36" ht="15">
@@ -6030,22 +6069,22 @@
         <v>51</v>
       </c>
       <c r="E36" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="F36" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>50</v>
       </c>
       <c r="H36" s="6">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="I36" s="6">
-        <v>7.6</v>
+        <v>0</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>326</v>
+        <v>50</v>
       </c>
       <c r="K36" t="s">
         <v>55</v>
@@ -6054,10 +6093,10 @@
         <v>0</v>
       </c>
       <c r="M36" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="N36" s="5" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="O36" s="6">
         <v>0</v>
@@ -6066,19 +6105,19 @@
         <v>57</v>
       </c>
       <c r="Q36" s="9" t="s">
-        <v>58</v>
+        <v>257</v>
       </c>
       <c r="R36" s="5" t="s">
         <v>59</v>
       </c>
       <c r="S36" s="6">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="T36" s="6">
-        <v>66.2</v>
+        <v>0.4</v>
       </c>
       <c r="U36" s="6">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="V36" t="s">
         <v>60</v>
@@ -6105,43 +6144,40 @@
         <v>1</v>
       </c>
       <c r="AH36" s="6">
-        <v>29.75</v>
+        <v>41.65</v>
       </c>
       <c r="AI36" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AM36" s="6">
-        <v>0</v>
-      </c>
       <c r="AN36" s="6">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="AO36" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="AP36" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AQ36" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR36" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS36" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="AT36" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="AU36" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="AV36" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="AW36" s="9" t="s">
         <v>327</v>
-      </c>
-      <c r="AP36" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AQ36" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR36" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS36" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="AT36" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="AU36" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="AV36" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="AW36" s="9" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="37" ht="15">
@@ -6149,16 +6185,16 @@
         <v>50</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>333</v>
+        <v>50</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>51</v>
       </c>
       <c r="E37" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="F37" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>50</v>
@@ -6167,40 +6203,46 @@
         <v>0</v>
       </c>
       <c r="I37" s="6">
-        <v>18.6</v>
+        <v>0</v>
       </c>
       <c r="J37" s="5" t="s">
         <v>50</v>
       </c>
       <c r="K37" t="s">
+        <v>55</v>
+      </c>
+      <c r="L37" s="7">
+        <v>0</v>
+      </c>
+      <c r="M37" t="s">
+        <v>328</v>
+      </c>
+      <c r="N37" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="O37" s="6">
+        <v>0</v>
+      </c>
+      <c r="P37" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q37" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="R37" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="S37" s="6">
+        <v>0</v>
+      </c>
+      <c r="T37" s="6">
+        <v>0</v>
+      </c>
+      <c r="U37" s="6">
+        <v>0</v>
+      </c>
+      <c r="V37" t="s">
         <v>60</v>
-      </c>
-      <c r="L37" s="7">
-        <v>0</v>
-      </c>
-      <c r="M37" t="s">
-        <v>334</v>
-      </c>
-      <c r="N37" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="O37" s="6">
-        <v>0</v>
-      </c>
-      <c r="P37" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="Q37" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="R37" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="S37" s="6">
-        <v>0</v>
-      </c>
-      <c r="V37" t="s">
-        <v>55</v>
       </c>
       <c r="W37" s="6">
         <v>0</v>
@@ -6233,31 +6275,31 @@
         <v>25</v>
       </c>
       <c r="AO37" s="5" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="AP37" s="5" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="AQ37" s="5" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="AR37" s="5" t="s">
         <v>50</v>
       </c>
       <c r="AS37" s="5" t="s">
-        <v>199</v>
+        <v>332</v>
       </c>
       <c r="AT37" s="5" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="AU37" s="5" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="AV37" s="5" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="AW37" s="9" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
     </row>
     <row r="38" ht="15">
@@ -6271,22 +6313,22 @@
         <v>51</v>
       </c>
       <c r="E38" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="F38" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>50</v>
       </c>
       <c r="H38" s="6">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="I38" s="6">
-        <v>9.5</v>
+        <v>7.6</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>50</v>
+        <v>339</v>
       </c>
       <c r="K38" t="s">
         <v>55</v>
@@ -6295,28 +6337,31 @@
         <v>0</v>
       </c>
       <c r="M38" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="N38" s="5" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="O38" s="6">
         <v>0</v>
       </c>
       <c r="P38" s="9" t="s">
-        <v>335</v>
+        <v>57</v>
       </c>
       <c r="Q38" s="9" t="s">
-        <v>165</v>
+        <v>58</v>
       </c>
       <c r="R38" s="5" t="s">
-        <v>336</v>
+        <v>59</v>
       </c>
       <c r="S38" s="6">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="T38" s="6">
-        <v>62.2</v>
+        <v>66.2</v>
+      </c>
+      <c r="U38" s="6">
+        <v>20</v>
       </c>
       <c r="V38" t="s">
         <v>60</v>
@@ -6343,40 +6388,43 @@
         <v>1</v>
       </c>
       <c r="AH38" s="6">
-        <v>20.83</v>
+        <v>29.75</v>
       </c>
       <c r="AI38" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="AM38" s="6">
+        <v>0</v>
+      </c>
       <c r="AN38" s="6">
-        <v>17.5</v>
+        <v>25</v>
       </c>
       <c r="AO38" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="AP38" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ38" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR38" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS38" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="AT38" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="AU38" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="AV38" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="AW38" s="9" t="s">
         <v>345</v>
-      </c>
-      <c r="AP38" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="AQ38" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR38" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS38" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="AT38" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="AU38" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="AV38" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="AW38" s="9" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="39" ht="15">
@@ -6384,16 +6432,16 @@
         <v>50</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>50</v>
+        <v>346</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>51</v>
       </c>
       <c r="E39" t="s">
-        <v>68</v>
+        <v>347</v>
       </c>
       <c r="F39" t="s">
-        <v>68</v>
+        <v>347</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>50</v>
@@ -6402,34 +6450,34 @@
         <v>0</v>
       </c>
       <c r="I39" s="6">
-        <v>0</v>
+        <v>18.6</v>
       </c>
       <c r="J39" s="5" t="s">
         <v>50</v>
       </c>
       <c r="K39" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="L39" s="7">
         <v>0</v>
       </c>
       <c r="M39" t="s">
-        <v>68</v>
+        <v>347</v>
       </c>
       <c r="N39" s="5" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="O39" s="6">
         <v>0</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>57</v>
+        <v>348</v>
       </c>
       <c r="Q39" s="9" t="s">
-        <v>58</v>
+        <v>209</v>
       </c>
       <c r="R39" s="5" t="s">
-        <v>59</v>
+        <v>349</v>
       </c>
       <c r="S39" s="6">
         <v>0</v>
@@ -6456,46 +6504,43 @@
         <v>1</v>
       </c>
       <c r="AC39" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH39" s="6">
-        <v>20.83</v>
+        <v>29.75</v>
       </c>
       <c r="AI39" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AM39" s="6">
-        <v>0</v>
-      </c>
       <c r="AN39" s="6">
-        <v>17.5</v>
+        <v>25</v>
       </c>
       <c r="AO39" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="AP39" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="AP39" s="5" t="s">
+      <c r="AQ39" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR39" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS39" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="AT39" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="AQ39" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AR39" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS39" s="5" t="s">
+      <c r="AU39" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="AT39" s="5" t="s">
+      <c r="AV39" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="AU39" s="5" t="s">
+      <c r="AW39" s="9" t="s">
         <v>355</v>
-      </c>
-      <c r="AV39" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="AW39" s="9" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="40" ht="15">
@@ -6509,10 +6554,10 @@
         <v>51</v>
       </c>
       <c r="E40" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="F40" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>50</v>
@@ -6521,10 +6566,10 @@
         <v>0</v>
       </c>
       <c r="I40" s="6">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>359</v>
+        <v>50</v>
       </c>
       <c r="K40" t="s">
         <v>55</v>
@@ -6533,31 +6578,28 @@
         <v>0</v>
       </c>
       <c r="M40" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="N40" s="5" t="s">
-        <v>56</v>
+        <v>177</v>
       </c>
       <c r="O40" s="6">
         <v>0</v>
       </c>
       <c r="P40" s="9" t="s">
-        <v>57</v>
+        <v>348</v>
       </c>
       <c r="Q40" s="9" t="s">
-        <v>58</v>
+        <v>178</v>
       </c>
       <c r="R40" s="5" t="s">
-        <v>59</v>
+        <v>349</v>
       </c>
       <c r="S40" s="6">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="T40" s="6">
-        <v>0</v>
-      </c>
-      <c r="U40" s="6">
-        <v>0</v>
+        <v>62.2</v>
       </c>
       <c r="V40" t="s">
         <v>60</v>
@@ -6584,43 +6626,40 @@
         <v>1</v>
       </c>
       <c r="AH40" s="6">
-        <v>148.75</v>
+        <v>20.83</v>
       </c>
       <c r="AI40" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AM40" s="6">
-        <v>0</v>
-      </c>
       <c r="AN40" s="6">
-        <v>125</v>
+        <v>17.5</v>
       </c>
       <c r="AO40" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="AP40" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="AQ40" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR40" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS40" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="AT40" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="AP40" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AQ40" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AR40" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS40" s="5" t="s">
+      <c r="AU40" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="AT40" s="5" t="s">
+      <c r="AV40" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="AU40" s="5" t="s">
+      <c r="AW40" s="9" t="s">
         <v>363</v>
-      </c>
-      <c r="AV40" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="AW40" s="9" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="41" ht="15">
@@ -6634,10 +6673,10 @@
         <v>51</v>
       </c>
       <c r="E41" t="s">
-        <v>366</v>
+        <v>52</v>
       </c>
       <c r="F41" t="s">
-        <v>366</v>
+        <v>52</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>50</v>
@@ -6649,7 +6688,7 @@
         <v>0</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>367</v>
+        <v>50</v>
       </c>
       <c r="K41" t="s">
         <v>55</v>
@@ -6658,10 +6697,10 @@
         <v>0</v>
       </c>
       <c r="M41" t="s">
-        <v>366</v>
+        <v>52</v>
       </c>
       <c r="N41" s="5" t="s">
-        <v>56</v>
+        <v>177</v>
       </c>
       <c r="O41" s="6">
         <v>0</v>
@@ -6678,14 +6717,8 @@
       <c r="S41" s="6">
         <v>0</v>
       </c>
-      <c r="T41" s="6">
-        <v>0</v>
-      </c>
-      <c r="U41" s="6">
-        <v>0</v>
-      </c>
       <c r="V41" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="W41" s="6">
         <v>0</v>
@@ -6706,10 +6739,10 @@
         <v>1</v>
       </c>
       <c r="AC41" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH41" s="6">
-        <v>29.75</v>
+        <v>20.83</v>
       </c>
       <c r="AI41" s="5" t="s">
         <v>50</v>
@@ -6718,34 +6751,34 @@
         <v>0</v>
       </c>
       <c r="AN41" s="6">
-        <v>25</v>
+        <v>17.5</v>
       </c>
       <c r="AO41" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="AP41" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="AQ41" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR41" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS41" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="AT41" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="AU41" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="AP41" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AQ41" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AR41" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS41" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="AT41" s="5" t="s">
+      <c r="AV41" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="AU41" s="5" t="s">
+      <c r="AW41" s="9" t="s">
         <v>370</v>
-      </c>
-      <c r="AV41" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="AW41" s="9" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="42" ht="15">
@@ -6759,10 +6792,10 @@
         <v>51</v>
       </c>
       <c r="E42" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="F42" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>50</v>
@@ -6771,10 +6804,10 @@
         <v>0</v>
       </c>
       <c r="I42" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="K42" t="s">
         <v>55</v>
@@ -6783,7 +6816,7 @@
         <v>0</v>
       </c>
       <c r="M42" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="N42" s="5" t="s">
         <v>56</v>
@@ -6795,7 +6828,7 @@
         <v>57</v>
       </c>
       <c r="Q42" s="9" t="s">
-        <v>376</v>
+        <v>58</v>
       </c>
       <c r="R42" s="5" t="s">
         <v>59</v>
@@ -6804,7 +6837,7 @@
         <v>0</v>
       </c>
       <c r="T42" s="6">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="U42" s="6">
         <v>0</v>
@@ -6834,7 +6867,7 @@
         <v>1</v>
       </c>
       <c r="AH42" s="6">
-        <v>29.75</v>
+        <v>148.75</v>
       </c>
       <c r="AI42" s="5" t="s">
         <v>50</v>
@@ -6843,13 +6876,13 @@
         <v>0</v>
       </c>
       <c r="AN42" s="6">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="AO42" s="5" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="AP42" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ42" s="5" t="s">
         <v>63</v>
@@ -6858,19 +6891,19 @@
         <v>50</v>
       </c>
       <c r="AS42" s="5" t="s">
-        <v>87</v>
+        <v>374</v>
       </c>
       <c r="AT42" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="AU42" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="AV42" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="AW42" s="9" t="s">
         <v>378</v>
-      </c>
-      <c r="AU42" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="AV42" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="AW42" s="9" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="43" ht="15">
@@ -6884,10 +6917,10 @@
         <v>51</v>
       </c>
       <c r="E43" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="F43" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>50</v>
@@ -6896,10 +6929,10 @@
         <v>0</v>
       </c>
       <c r="I43" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="K43" t="s">
         <v>55</v>
@@ -6908,7 +6941,7 @@
         <v>0</v>
       </c>
       <c r="M43" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="N43" s="5" t="s">
         <v>56</v>
@@ -6920,7 +6953,7 @@
         <v>57</v>
       </c>
       <c r="Q43" s="9" t="s">
-        <v>376</v>
+        <v>58</v>
       </c>
       <c r="R43" s="5" t="s">
         <v>59</v>
@@ -6959,7 +6992,7 @@
         <v>1</v>
       </c>
       <c r="AH43" s="6">
-        <v>148.75</v>
+        <v>29.75</v>
       </c>
       <c r="AI43" s="5" t="s">
         <v>50</v>
@@ -6968,13 +7001,13 @@
         <v>0</v>
       </c>
       <c r="AN43" s="6">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AO43" s="5" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="AP43" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="AQ43" s="5" t="s">
         <v>63</v>
@@ -6983,19 +7016,19 @@
         <v>50</v>
       </c>
       <c r="AS43" s="5" t="s">
-        <v>95</v>
+        <v>138</v>
       </c>
       <c r="AT43" s="5" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="AU43" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="AV43" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="AW43" s="9" t="s">
         <v>385</v>
-      </c>
-      <c r="AV43" s="5" t="s">
-        <v>386</v>
-      </c>
-      <c r="AW43" s="9" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="44" ht="15">
@@ -7009,10 +7042,10 @@
         <v>51</v>
       </c>
       <c r="E44" t="s">
-        <v>68</v>
+        <v>386</v>
       </c>
       <c r="F44" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>50</v>
@@ -7021,10 +7054,10 @@
         <v>0</v>
       </c>
       <c r="I44" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="K44" t="s">
         <v>55</v>
@@ -7045,7 +7078,7 @@
         <v>57</v>
       </c>
       <c r="Q44" s="9" t="s">
-        <v>58</v>
+        <v>389</v>
       </c>
       <c r="R44" s="5" t="s">
         <v>59</v>
@@ -7054,6 +7087,9 @@
         <v>0</v>
       </c>
       <c r="T44" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="U44" s="6">
         <v>0</v>
       </c>
       <c r="V44" t="s">
@@ -7081,7 +7117,7 @@
         <v>1</v>
       </c>
       <c r="AH44" s="6">
-        <v>131.5</v>
+        <v>29.75</v>
       </c>
       <c r="AI44" s="5" t="s">
         <v>50</v>
@@ -7090,34 +7126,281 @@
         <v>0</v>
       </c>
       <c r="AN44" s="6">
-        <v>110.5</v>
+        <v>25</v>
       </c>
       <c r="AO44" s="5" t="s">
         <v>390</v>
       </c>
       <c r="AP44" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ44" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR44" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS44" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AT44" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="AQ44" s="5" t="s">
+      <c r="AU44" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="AR44" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS44" s="5" t="s">
+      <c r="AV44" s="5" t="s">
         <v>393</v>
       </c>
-      <c r="AT44" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AU44" s="5" t="s">
+      <c r="AW44" s="9" t="s">
         <v>394</v>
       </c>
-      <c r="AV44" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="AW44" s="9" t="s">
+    </row>
+    <row r="45" ht="15">
+      <c r="B45" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E45" t="s">
         <v>395</v>
+      </c>
+      <c r="F45" t="s">
+        <v>395</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H45" s="6">
+        <v>0</v>
+      </c>
+      <c r="I45" s="6">
+        <v>1</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="K45" t="s">
+        <v>55</v>
+      </c>
+      <c r="L45" s="7">
+        <v>0</v>
+      </c>
+      <c r="M45" t="s">
+        <v>395</v>
+      </c>
+      <c r="N45" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="O45" s="6">
+        <v>0</v>
+      </c>
+      <c r="P45" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q45" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="R45" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="S45" s="6">
+        <v>0</v>
+      </c>
+      <c r="T45" s="6">
+        <v>0</v>
+      </c>
+      <c r="U45" s="6">
+        <v>0</v>
+      </c>
+      <c r="V45" t="s">
+        <v>60</v>
+      </c>
+      <c r="W45" s="6">
+        <v>0</v>
+      </c>
+      <c r="X45" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y45" s="7">
+        <v>1</v>
+      </c>
+      <c r="Z45" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA45" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB45" s="7">
+        <v>1</v>
+      </c>
+      <c r="AC45" s="7">
+        <v>1</v>
+      </c>
+      <c r="AH45" s="6">
+        <v>148.75</v>
+      </c>
+      <c r="AI45" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AM45" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN45" s="6">
+        <v>125</v>
+      </c>
+      <c r="AO45" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="AP45" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ45" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR45" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS45" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="AT45" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="AU45" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="AV45" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="AW45" s="9" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="46" ht="15">
+      <c r="B46" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E46" t="s">
+        <v>52</v>
+      </c>
+      <c r="F46" t="s">
+        <v>401</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H46" s="6">
+        <v>0</v>
+      </c>
+      <c r="I46" s="6">
+        <v>0</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>402</v>
+      </c>
+      <c r="K46" t="s">
+        <v>55</v>
+      </c>
+      <c r="L46" s="7">
+        <v>0</v>
+      </c>
+      <c r="M46" t="s">
+        <v>401</v>
+      </c>
+      <c r="N46" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="O46" s="6">
+        <v>0</v>
+      </c>
+      <c r="P46" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q46" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="R46" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="S46" s="6">
+        <v>0</v>
+      </c>
+      <c r="T46" s="6">
+        <v>0</v>
+      </c>
+      <c r="V46" t="s">
+        <v>60</v>
+      </c>
+      <c r="W46" s="6">
+        <v>0</v>
+      </c>
+      <c r="X46" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y46" s="7">
+        <v>1</v>
+      </c>
+      <c r="Z46" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA46" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB46" s="7">
+        <v>1</v>
+      </c>
+      <c r="AC46" s="7">
+        <v>1</v>
+      </c>
+      <c r="AH46" s="6">
+        <v>131.5</v>
+      </c>
+      <c r="AI46" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AM46" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN46" s="6">
+        <v>110.5</v>
+      </c>
+      <c r="AO46" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="AP46" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="AQ46" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="AR46" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS46" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="AT46" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AU46" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="AV46" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="AW46" s="9" t="s">
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>